<commit_message>
Adicionado testes 2: wedos_test_pool
</commit_message>
<xml_diff>
--- a/experiment_results/combined_sweep/rtt_bursts_S1_atk10pct_wu300000.xlsx
+++ b/experiment_results/combined_sweep/rtt_bursts_S1_atk10pct_wu300000.xlsx
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>00:010.0</t>
+          <t>00:010.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -486,12 +486,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>18.9</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -533,27 +533,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>00:020.2</t>
+          <t>00:020.5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>22.1</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>26.8</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9.43</t>
+          <t>23.66</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1040</t>
+          <t>9690</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -583,34 +583,34 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>00:030.0</t>
+          <t>00:029.9</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>24.3</t>
+          <t>38.1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27.8</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6.40</t>
+          <t>8.28</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>21393</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -640,34 +640,34 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>00:040.2</t>
+          <t>00:040.1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>22.7</t>
+          <t>33.9</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3.61</t>
+          <t>3.58</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22923</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -709,22 +709,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.5</t>
+          <t>27.2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>22.5</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.09</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4.64</t>
+          <t>6.53</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>24587</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -761,27 +761,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:000.1</t>
+          <t>00:059.8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>19.8</t>
+          <t>40.8</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23.0</t>
+          <t>50.9</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.14</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4.82</t>
+          <t>10.11</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -801,44 +801,44 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>38509</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01:009.8</t>
+          <t>01:010.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>21.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23.1</t>
+          <t>94.9</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4.71</t>
+          <t>10.44</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -858,17 +858,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>79993</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
@@ -880,22 +880,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>21.3</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>100.1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5.74</t>
+          <t>5.28</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -915,44 +915,44 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>117818</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>01:030.1</t>
+          <t>01:029.9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>38.1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23.6</t>
+          <t>61.6</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -962,17 +962,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5.62</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>128894</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -982,34 +982,34 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>01:039.8</t>
+          <t>01:039.7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>22.9</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>5.93</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1029,12 +1029,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>130212</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1046,27 +1046,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>01:050.0</t>
+          <t>01:050.2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>20.3</t>
+          <t>21.4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23.1</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5.16</t>
+          <t>4.24</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1086,12 +1086,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>126897</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1108,12 +1108,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>24.6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23.0</t>
+          <t>32.1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>8.24</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1143,12 +1143,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>126227</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1160,27 +1160,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>02:009.9</t>
+          <t>02:010.2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>27.4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23.6</t>
+          <t>34.1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4.60</t>
+          <t>6.57</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>127979</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1217,27 +1217,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>02:020.3</t>
+          <t>02:020.0</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23.9</t>
+          <t>43.1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4.47</t>
+          <t>9.55</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1257,44 +1257,44 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>133733</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>02:029.7</t>
+          <t>02:030.0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>19.5</t>
+          <t>33.4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23.0</t>
+          <t>44.8</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>7.45</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1314,17 +1314,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>140797</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Normal/Residual</t>
+          <t>DDoS Burst</t>
         </is>
       </c>
     </row>
@@ -1336,22 +1336,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>17.3</t>
+          <t>24.0</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>21.1</t>
+          <t>30.4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1361,22 +1361,22 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>3.14</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>139619</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1388,27 +1388,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>02:050.2</t>
+          <t>02:050.1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>17.3</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>133266</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1445,27 +1445,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>02:055.0</t>
+          <t>02:055.2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>2.48</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1485,12 +1485,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>130147</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">

</xml_diff>